<commit_message>
-> Wir haben erstmal weitere Fehlermeldung ccode im main (use_case.py) geschreiben uum erstmal welche zu haben
-> bei den produktions_manger haben wir für den use case den funktion geschreibe des logbuch eintrags in der datenbank so das es die daten gespeichert werden könnte
-> dann eine weiter Funktion im Produktions_manbger wo wir in der funktion halt wenn die maschine repariert ist und der status wieder auf Aktiv muss das ticket geschlossen werden
</commit_message>
<xml_diff>
--- a/Mitarbeiter/Alle_Bestande_nach_Lagerort.xlsx
+++ b/Mitarbeiter/Alle_Bestande_nach_Lagerort.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,198 +464,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AT.045</t>
+          <t>DE309012</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ÖL</t>
+          <t>Cement säcke</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Schmierstoffe</t>
+          <t>cement</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lieter</t>
+          <t>Stück</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>30</v>
+        <v>5.06</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Hamburg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>T05679</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Edelstrahl Quadratrohr 15X15X1,5mm 500mm</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Edelstahl Rohre</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Hamburg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>B004567</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Stahlblech 2x2M</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Bleche</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Hamburg</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Df23123</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Stahlschraube Stahlschrauben 4 x 25 mm</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Schrauben Flugzeug</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Hamburg</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DK2350</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Blechschrauben DIN 7072 - 3,6 mm - Senkkopf - Schlitz - A2</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Schrauben</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Hamburg</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>DN00789</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bohrschrauben DIN 7504M-H Rundkopf schwarz verzinkt 4,2x22 </t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Schrauben</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Hamburg</t>
+          <t>Lemgo</t>
         </is>
       </c>
     </row>

</xml_diff>